<commit_message>
Update TestRunner to JUnit 4, sequential execution order, fix HomeLoan header mismatch, and package latest ZIP
</commit_message>
<xml_diff>
--- a/UI_Validation_Results.xlsx
+++ b/UI_Validation_Results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="25">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -29,55 +29,55 @@
     <t>Status</t>
   </si>
   <si>
+    <t>EMI Calculator</t>
+  </si>
+  <si>
+    <t>Loan Amount</t>
+  </si>
+  <si>
+    <t>1500000</t>
+  </si>
+  <si>
+    <t>15,00,000</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>Interest Rate</t>
+  </si>
+  <si>
+    <t>9.5</t>
+  </si>
+  <si>
+    <t>Loan Term</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Years</t>
+  </si>
+  <si>
+    <t>Monthly EMI</t>
+  </si>
+  <si>
+    <t>131525</t>
+  </si>
+  <si>
+    <t>1,31,525.27</t>
+  </si>
+  <si>
     <t>Loan Amount Calculator</t>
   </si>
   <si>
-    <t>Monthly EMI</t>
-  </si>
-  <si>
-    <t>131525</t>
-  </si>
-  <si>
     <t>1,31,525.00</t>
   </si>
   <si>
-    <t>PASS</t>
-  </si>
-  <si>
-    <t>Interest Rate</t>
-  </si>
-  <si>
-    <t>9.5</t>
-  </si>
-  <si>
-    <t>Loan Term</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Years</t>
-  </si>
-  <si>
     <t>Total Loan Amount</t>
   </si>
   <si>
-    <t>1500000</t>
-  </si>
-  <si>
     <t>14,99,997</t>
-  </si>
-  <si>
-    <t>EMI Calculator</t>
-  </si>
-  <si>
-    <t>Loan Amount</t>
-  </si>
-  <si>
-    <t>15,00,000</t>
-  </si>
-  <si>
-    <t>1,31,525.27</t>
   </si>
   <si>
     <t>Loan Tenure Calculator</t>
@@ -181,7 +181,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="20.2734375" customWidth="true" bestFit="true"/>
@@ -298,13 +298,13 @@
         <v>18</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s" s="0">
         <v>16</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E7" t="s" s="2">
         <v>9</v>
@@ -366,7 +366,7 @@
         <v>18</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s" s="0">
         <v>7</v>
@@ -383,13 +383,13 @@
         <v>22</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E12" t="s" s="2">
         <v>9</v>
@@ -400,13 +400,13 @@
         <v>22</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E13" t="s" s="2">
         <v>9</v>
@@ -443,244 +443,6 @@
         <v>24</v>
       </c>
       <c r="E15" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="B16" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="C16" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D16" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E16" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="B17" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="C17" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D17" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="E17" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="B18" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="C18" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="D18" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="E18" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="B19" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="C19" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="D19" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="E19" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="B20" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="C20" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D20" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E20" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="B21" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="C21" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="D21" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="E21" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="B22" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C22" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D22" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="E22" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="B23" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C23" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="D23" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E23" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="B24" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="C24" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D24" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E24" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="B25" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="C25" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D25" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="E25" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="B26" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="C26" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="D26" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="E26" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="B27" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C27" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D27" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="E27" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="B28" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C28" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="D28" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E28" t="s" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="B29" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="C29" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D29" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="E29" t="s" s="2">
         <v>9</v>
       </c>
     </row>

</xml_diff>